<commit_message>
AlgList UPD 2026-01-16 10:01
</commit_message>
<xml_diff>
--- a/SkienAlgsListFinal.xlsx
+++ b/SkienAlgsListFinal.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr codeName="ЭтаКнига"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://urfume-my.sharepoint.com/personal/sergey_osipov_urfu_me/Documents/AiSD2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1241" documentId="13_ncr:1_{BB64072A-02B6-4C3F-B1E2-71C6B558E3EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{52E0DE3F-A1D1-4E0B-A8DB-70F09B1A2028}"/>
+  <xr:revisionPtr revIDLastSave="1242" documentId="13_ncr:1_{BB64072A-02B6-4C3F-B1E2-71C6B558E3EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9157DA7B-2BA9-4A33-8F18-DAB71EFADF0E}"/>
   <bookViews>
-    <workbookView xWindow="-270" yWindow="900" windowWidth="22080" windowHeight="12210" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2295" yWindow="780" windowWidth="18570" windowHeight="14550" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191028" refMode="R1C1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -2585,19 +2585,19 @@
       </c>
     </row>
     <row r="19" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="14" t="s">
+      <c r="A19" s="35" t="s">
         <v>70</v>
       </c>
-      <c r="B19" s="14" t="s">
+      <c r="B19" s="35" t="s">
         <v>79</v>
       </c>
-      <c r="C19" s="14" t="s">
+      <c r="C19" s="35" t="s">
         <v>80</v>
       </c>
-      <c r="D19" s="14">
+      <c r="D19" s="35">
         <v>148</v>
       </c>
-      <c r="E19" s="14">
+      <c r="E19" s="35">
         <v>4</v>
       </c>
       <c r="F19" s="17" t="s">
@@ -2621,19 +2621,19 @@
       </c>
     </row>
     <row r="20" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="14" t="s">
+      <c r="A20" s="35" t="s">
         <v>82</v>
       </c>
-      <c r="B20" s="14" t="s">
+      <c r="B20" s="35" t="s">
         <v>83</v>
       </c>
-      <c r="C20" s="14" t="s">
+      <c r="C20" s="35" t="s">
         <v>84</v>
       </c>
-      <c r="D20" s="14">
+      <c r="D20" s="35">
         <v>148</v>
       </c>
-      <c r="E20" s="14">
+      <c r="E20" s="35">
         <v>9</v>
       </c>
       <c r="F20" s="17" t="s">
@@ -2657,19 +2657,19 @@
       </c>
     </row>
     <row r="21" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="14" t="s">
+      <c r="A21" s="35" t="s">
         <v>86</v>
       </c>
-      <c r="B21" s="14" t="s">
+      <c r="B21" s="35" t="s">
         <v>87</v>
       </c>
-      <c r="C21" s="14" t="s">
+      <c r="C21" s="35" t="s">
         <v>88</v>
       </c>
-      <c r="D21" s="14">
+      <c r="D21" s="35">
         <v>150</v>
       </c>
-      <c r="E21" s="14">
+      <c r="E21" s="35">
         <v>18</v>
       </c>
       <c r="F21" s="17" t="s">
@@ -2693,19 +2693,19 @@
       </c>
     </row>
     <row r="22" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="14" t="s">
+      <c r="A22" s="35" t="s">
         <v>89</v>
       </c>
-      <c r="B22" s="14" t="s">
+      <c r="B22" s="35" t="s">
         <v>90</v>
       </c>
-      <c r="C22" s="14" t="s">
+      <c r="C22" s="35" t="s">
         <v>91</v>
       </c>
-      <c r="D22" s="14">
+      <c r="D22" s="35">
         <v>150</v>
       </c>
-      <c r="E22" s="14">
+      <c r="E22" s="35">
         <v>10</v>
       </c>
       <c r="F22" s="17" t="s">

</xml_diff>